<commit_message>
Adjustment of the Boltzmann model
</commit_message>
<xml_diff>
--- a/LineClass/chance_mc_summary.xlsx
+++ b/LineClass/chance_mc_summary.xlsx
@@ -493,43 +493,43 @@
         <v>-11.3</v>
       </c>
       <c r="B2" t="n">
-        <v>2982</v>
+        <v>5015</v>
       </c>
       <c r="C2" t="n">
-        <v>1413</v>
+        <v>1198</v>
       </c>
       <c r="D2" t="n">
-        <v>1413</v>
+        <v>1198</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="G2" t="n">
-        <v>61</v>
+        <v>91</v>
       </c>
       <c r="H2" t="n">
-        <v>80</v>
+        <v>111</v>
       </c>
       <c r="I2" t="n">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="J2" t="n">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="K2" t="n">
-        <v>62</v>
+        <v>45</v>
       </c>
       <c r="L2" t="n">
-        <v>46</v>
+        <v>26</v>
       </c>
       <c r="M2" t="n">
-        <v>103</v>
+        <v>67</v>
       </c>
       <c r="N2" t="n">
-        <v>0.03</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="3">
@@ -537,43 +537,43 @@
         <v>-9.699999999999999</v>
       </c>
       <c r="B3" t="n">
-        <v>3110</v>
+        <v>4963</v>
       </c>
       <c r="C3" t="n">
-        <v>1551</v>
+        <v>1227</v>
       </c>
       <c r="D3" t="n">
-        <v>1551</v>
+        <v>1227</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>41</v>
+        <v>63</v>
       </c>
       <c r="G3" t="n">
-        <v>51</v>
+        <v>107</v>
       </c>
       <c r="H3" t="n">
-        <v>71</v>
+        <v>106</v>
       </c>
       <c r="I3" t="n">
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="J3" t="n">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="K3" t="n">
-        <v>69</v>
+        <v>43</v>
       </c>
       <c r="L3" t="n">
-        <v>55</v>
+        <v>31</v>
       </c>
       <c r="M3" t="n">
-        <v>122</v>
+        <v>70</v>
       </c>
       <c r="N3" t="n">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="4">
@@ -581,43 +581,43 @@
         <v>-8.300000000000001</v>
       </c>
       <c r="B4" t="n">
-        <v>2988</v>
+        <v>5045</v>
       </c>
       <c r="C4" t="n">
-        <v>1462</v>
+        <v>1250</v>
       </c>
       <c r="D4" t="n">
-        <v>1462</v>
+        <v>1250</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="G4" t="n">
-        <v>58</v>
+        <v>92</v>
       </c>
       <c r="H4" t="n">
-        <v>71</v>
+        <v>121</v>
       </c>
       <c r="I4" t="n">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="J4" t="n">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="K4" t="n">
+        <v>52</v>
+      </c>
+      <c r="L4" t="n">
+        <v>34</v>
+      </c>
+      <c r="M4" t="n">
         <v>64</v>
       </c>
-      <c r="L4" t="n">
-        <v>49</v>
-      </c>
-      <c r="M4" t="n">
-        <v>105</v>
-      </c>
       <c r="N4" t="n">
-        <v>0.03</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="5">
@@ -625,43 +625,43 @@
         <v>-6.9</v>
       </c>
       <c r="B5" t="n">
-        <v>2995</v>
+        <v>5303</v>
       </c>
       <c r="C5" t="n">
-        <v>1452</v>
+        <v>1303</v>
       </c>
       <c r="D5" t="n">
-        <v>1452</v>
+        <v>1303</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="G5" t="n">
-        <v>62</v>
+        <v>85</v>
       </c>
       <c r="H5" t="n">
-        <v>85</v>
+        <v>126</v>
       </c>
       <c r="I5" t="n">
-        <v>72</v>
+        <v>126</v>
       </c>
       <c r="J5" t="n">
-        <v>83</v>
+        <v>58</v>
       </c>
       <c r="K5" t="n">
-        <v>62</v>
+        <v>39</v>
       </c>
       <c r="L5" t="n">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="M5" t="n">
-        <v>109</v>
+        <v>74</v>
       </c>
       <c r="N5" t="n">
-        <v>0.04</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="6">
@@ -669,43 +669,43 @@
         <v>6.9</v>
       </c>
       <c r="B6" t="n">
-        <v>3005</v>
+        <v>4991</v>
       </c>
       <c r="C6" t="n">
-        <v>1433</v>
+        <v>1207</v>
       </c>
       <c r="D6" t="n">
-        <v>1433</v>
+        <v>1207</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="G6" t="n">
-        <v>54</v>
+        <v>102</v>
       </c>
       <c r="H6" t="n">
+        <v>116</v>
+      </c>
+      <c r="I6" t="n">
+        <v>85</v>
+      </c>
+      <c r="J6" t="n">
+        <v>55</v>
+      </c>
+      <c r="K6" t="n">
+        <v>40</v>
+      </c>
+      <c r="L6" t="n">
+        <v>36</v>
+      </c>
+      <c r="M6" t="n">
         <v>74</v>
       </c>
-      <c r="I6" t="n">
-        <v>81</v>
-      </c>
-      <c r="J6" t="n">
-        <v>77</v>
-      </c>
-      <c r="K6" t="n">
-        <v>56</v>
-      </c>
-      <c r="L6" t="n">
-        <v>55</v>
-      </c>
-      <c r="M6" t="n">
-        <v>103</v>
-      </c>
       <c r="N6" t="n">
-        <v>0.03</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="7">
@@ -713,43 +713,43 @@
         <v>8.300000000000001</v>
       </c>
       <c r="B7" t="n">
-        <v>3038</v>
+        <v>5116</v>
       </c>
       <c r="C7" t="n">
-        <v>1479</v>
+        <v>1254</v>
       </c>
       <c r="D7" t="n">
-        <v>1479</v>
+        <v>1254</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="G7" t="n">
-        <v>61</v>
+        <v>102</v>
       </c>
       <c r="H7" t="n">
-        <v>85</v>
+        <v>114</v>
       </c>
       <c r="I7" t="n">
-        <v>79</v>
+        <v>92</v>
       </c>
       <c r="J7" t="n">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="K7" t="n">
-        <v>56</v>
+        <v>36</v>
       </c>
       <c r="L7" t="n">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="M7" t="n">
-        <v>113</v>
+        <v>74</v>
       </c>
       <c r="N7" t="n">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="8">
@@ -757,43 +757,43 @@
         <v>9.699999999999999</v>
       </c>
       <c r="B8" t="n">
-        <v>2968</v>
+        <v>5139</v>
       </c>
       <c r="C8" t="n">
-        <v>1465</v>
+        <v>1233</v>
       </c>
       <c r="D8" t="n">
-        <v>1465</v>
+        <v>1233</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="G8" t="n">
-        <v>67</v>
+        <v>89</v>
       </c>
       <c r="H8" t="n">
-        <v>70</v>
+        <v>130</v>
       </c>
       <c r="I8" t="n">
-        <v>81</v>
+        <v>99</v>
       </c>
       <c r="J8" t="n">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="K8" t="n">
-        <v>68</v>
+        <v>30</v>
       </c>
       <c r="L8" t="n">
-        <v>48</v>
+        <v>31</v>
       </c>
       <c r="M8" t="n">
-        <v>115</v>
+        <v>79</v>
       </c>
       <c r="N8" t="n">
-        <v>0.04</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="9">
@@ -801,43 +801,43 @@
         <v>11.3</v>
       </c>
       <c r="B9" t="n">
-        <v>3037</v>
+        <v>4876</v>
       </c>
       <c r="C9" t="n">
-        <v>1454</v>
+        <v>1184</v>
       </c>
       <c r="D9" t="n">
-        <v>1454</v>
+        <v>1184</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>33</v>
+        <v>49</v>
       </c>
       <c r="G9" t="n">
-        <v>58</v>
+        <v>89</v>
       </c>
       <c r="H9" t="n">
-        <v>74</v>
+        <v>129</v>
       </c>
       <c r="I9" t="n">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="J9" t="n">
-        <v>78</v>
+        <v>61</v>
       </c>
       <c r="K9" t="n">
-        <v>59</v>
+        <v>41</v>
       </c>
       <c r="L9" t="n">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="M9" t="n">
-        <v>105</v>
+        <v>64</v>
       </c>
       <c r="N9" t="n">
-        <v>0.03</v>
+        <v>0.09</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Boltzmann iterations and LOPT corrections
</commit_message>
<xml_diff>
--- a/LineClass/chance_mc_summary.xlsx
+++ b/LineClass/chance_mc_summary.xlsx
@@ -493,43 +493,43 @@
         <v>-11.3</v>
       </c>
       <c r="B2" t="n">
-        <v>5015</v>
+        <v>4729</v>
       </c>
       <c r="C2" t="n">
-        <v>1198</v>
+        <v>1190</v>
       </c>
       <c r="D2" t="n">
-        <v>1198</v>
+        <v>1190</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>48</v>
+        <v>62</v>
       </c>
       <c r="G2" t="n">
-        <v>91</v>
+        <v>119</v>
       </c>
       <c r="H2" t="n">
         <v>111</v>
       </c>
       <c r="I2" t="n">
-        <v>96</v>
+        <v>78</v>
       </c>
       <c r="J2" t="n">
-        <v>73</v>
+        <v>56</v>
       </c>
       <c r="K2" t="n">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="L2" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="M2" t="n">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="N2" t="n">
-        <v>0.13</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="3">
@@ -537,43 +537,43 @@
         <v>-9.699999999999999</v>
       </c>
       <c r="B3" t="n">
-        <v>4963</v>
+        <v>4492</v>
       </c>
       <c r="C3" t="n">
-        <v>1227</v>
+        <v>1110</v>
       </c>
       <c r="D3" t="n">
-        <v>1227</v>
+        <v>1110</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>63</v>
+        <v>75</v>
       </c>
       <c r="G3" t="n">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="H3" t="n">
-        <v>106</v>
+        <v>117</v>
       </c>
       <c r="I3" t="n">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="J3" t="n">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="K3" t="n">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="L3" t="n">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="M3" t="n">
-        <v>70</v>
+        <v>48</v>
       </c>
       <c r="N3" t="n">
-        <v>0.1</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="4">
@@ -581,40 +581,40 @@
         <v>-8.300000000000001</v>
       </c>
       <c r="B4" t="n">
-        <v>5045</v>
+        <v>4693</v>
       </c>
       <c r="C4" t="n">
-        <v>1250</v>
+        <v>1167</v>
       </c>
       <c r="D4" t="n">
-        <v>1250</v>
+        <v>1167</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>42</v>
+        <v>68</v>
       </c>
       <c r="G4" t="n">
-        <v>92</v>
+        <v>106</v>
       </c>
       <c r="H4" t="n">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="I4" t="n">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="J4" t="n">
         <v>73</v>
       </c>
       <c r="K4" t="n">
-        <v>52</v>
+        <v>31</v>
       </c>
       <c r="L4" t="n">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="M4" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="N4" t="n">
         <v>0.11</v>
@@ -625,43 +625,43 @@
         <v>-6.9</v>
       </c>
       <c r="B5" t="n">
-        <v>5303</v>
+        <v>4869</v>
       </c>
       <c r="C5" t="n">
-        <v>1303</v>
+        <v>1235</v>
       </c>
       <c r="D5" t="n">
-        <v>1303</v>
+        <v>1235</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
+        <v>52</v>
+      </c>
+      <c r="G5" t="n">
+        <v>108</v>
+      </c>
+      <c r="H5" t="n">
+        <v>121</v>
+      </c>
+      <c r="I5" t="n">
+        <v>96</v>
+      </c>
+      <c r="J5" t="n">
+        <v>55</v>
+      </c>
+      <c r="K5" t="n">
+        <v>32</v>
+      </c>
+      <c r="L5" t="n">
         <v>36</v>
       </c>
-      <c r="G5" t="n">
-        <v>85</v>
-      </c>
-      <c r="H5" t="n">
-        <v>126</v>
-      </c>
-      <c r="I5" t="n">
-        <v>126</v>
-      </c>
-      <c r="J5" t="n">
-        <v>58</v>
-      </c>
-      <c r="K5" t="n">
-        <v>39</v>
-      </c>
-      <c r="L5" t="n">
-        <v>34</v>
-      </c>
       <c r="M5" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="N5" t="n">
-        <v>0.11</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="6">
@@ -669,43 +669,43 @@
         <v>6.9</v>
       </c>
       <c r="B6" t="n">
-        <v>4991</v>
+        <v>4676</v>
       </c>
       <c r="C6" t="n">
-        <v>1207</v>
+        <v>1142</v>
       </c>
       <c r="D6" t="n">
-        <v>1207</v>
+        <v>1142</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>42</v>
+        <v>59</v>
       </c>
       <c r="G6" t="n">
-        <v>102</v>
+        <v>126</v>
       </c>
       <c r="H6" t="n">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="I6" t="n">
         <v>85</v>
       </c>
       <c r="J6" t="n">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="K6" t="n">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="L6" t="n">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="M6" t="n">
-        <v>74</v>
+        <v>57</v>
       </c>
       <c r="N6" t="n">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="7">
@@ -713,43 +713,43 @@
         <v>8.300000000000001</v>
       </c>
       <c r="B7" t="n">
-        <v>5116</v>
+        <v>4797</v>
       </c>
       <c r="C7" t="n">
-        <v>1254</v>
+        <v>1195</v>
       </c>
       <c r="D7" t="n">
-        <v>1254</v>
+        <v>1195</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="G7" t="n">
-        <v>102</v>
+        <v>118</v>
       </c>
       <c r="H7" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="I7" t="n">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="J7" t="n">
-        <v>63</v>
+        <v>46</v>
       </c>
       <c r="K7" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="L7" t="n">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="M7" t="n">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="N7" t="n">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="8">
@@ -757,43 +757,43 @@
         <v>9.699999999999999</v>
       </c>
       <c r="B8" t="n">
-        <v>5139</v>
+        <v>4659</v>
       </c>
       <c r="C8" t="n">
-        <v>1233</v>
+        <v>1162</v>
       </c>
       <c r="D8" t="n">
-        <v>1233</v>
+        <v>1162</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>54</v>
+        <v>64</v>
       </c>
       <c r="G8" t="n">
-        <v>89</v>
+        <v>112</v>
       </c>
       <c r="H8" t="n">
-        <v>130</v>
+        <v>113</v>
       </c>
       <c r="I8" t="n">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="J8" t="n">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="K8" t="n">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="L8" t="n">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="M8" t="n">
-        <v>79</v>
+        <v>57</v>
       </c>
       <c r="N8" t="n">
-        <v>0.09</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="9">
@@ -801,43 +801,43 @@
         <v>11.3</v>
       </c>
       <c r="B9" t="n">
-        <v>4876</v>
+        <v>4618</v>
       </c>
       <c r="C9" t="n">
-        <v>1184</v>
+        <v>1176</v>
       </c>
       <c r="D9" t="n">
-        <v>1184</v>
+        <v>1176</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="G9" t="n">
-        <v>89</v>
+        <v>121</v>
       </c>
       <c r="H9" t="n">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="I9" t="n">
-        <v>103</v>
+        <v>84</v>
       </c>
       <c r="J9" t="n">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="K9" t="n">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="L9" t="n">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="M9" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="N9" t="n">
-        <v>0.09</v>
+        <v>0.11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
tools/estimate_snr.py, intensity calibration, etc.
line_decisions.csv ledger introduced, as well as new_levels.csv, icalc_new.csv, revised_levels.csv - to enable revision of old levels and search for new ones in conjunction with IDEN2 and LOPT.
</commit_message>
<xml_diff>
--- a/LineClass/chance_mc_summary.xlsx
+++ b/LineClass/chance_mc_summary.xlsx
@@ -493,40 +493,40 @@
         <v>-11.3</v>
       </c>
       <c r="B2" t="n">
-        <v>4729</v>
+        <v>4586</v>
       </c>
       <c r="C2" t="n">
-        <v>1190</v>
+        <v>1165</v>
       </c>
       <c r="D2" t="n">
-        <v>1190</v>
+        <v>1165</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="G2" t="n">
-        <v>119</v>
+        <v>137</v>
       </c>
       <c r="H2" t="n">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="I2" t="n">
         <v>78</v>
       </c>
       <c r="J2" t="n">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="K2" t="n">
         <v>37</v>
       </c>
       <c r="L2" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="M2" t="n">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="N2" t="n">
         <v>0.12</v>
@@ -537,43 +537,43 @@
         <v>-9.699999999999999</v>
       </c>
       <c r="B3" t="n">
-        <v>4492</v>
+        <v>4728</v>
       </c>
       <c r="C3" t="n">
-        <v>1110</v>
+        <v>1209</v>
       </c>
       <c r="D3" t="n">
-        <v>1110</v>
+        <v>1209</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="G3" t="n">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="H3" t="n">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="I3" t="n">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="J3" t="n">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="K3" t="n">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="L3" t="n">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="M3" t="n">
-        <v>48</v>
+        <v>63</v>
       </c>
       <c r="N3" t="n">
-        <v>0.13</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="4">
@@ -581,43 +581,43 @@
         <v>-8.300000000000001</v>
       </c>
       <c r="B4" t="n">
-        <v>4693</v>
+        <v>4631</v>
       </c>
       <c r="C4" t="n">
-        <v>1167</v>
+        <v>1243</v>
       </c>
       <c r="D4" t="n">
-        <v>1167</v>
+        <v>1243</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="G4" t="n">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="H4" t="n">
-        <v>126</v>
+        <v>111</v>
       </c>
       <c r="I4" t="n">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="J4" t="n">
-        <v>73</v>
+        <v>59</v>
       </c>
       <c r="K4" t="n">
-        <v>31</v>
+        <v>43</v>
       </c>
       <c r="L4" t="n">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="M4" t="n">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="N4" t="n">
-        <v>0.11</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="5">
@@ -625,43 +625,43 @@
         <v>-6.9</v>
       </c>
       <c r="B5" t="n">
-        <v>4869</v>
+        <v>4578</v>
       </c>
       <c r="C5" t="n">
-        <v>1235</v>
+        <v>1268</v>
       </c>
       <c r="D5" t="n">
-        <v>1235</v>
+        <v>1268</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="G5" t="n">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="H5" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="I5" t="n">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="J5" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="K5" t="n">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="L5" t="n">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="M5" t="n">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="N5" t="n">
-        <v>0.09</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="6">
@@ -669,43 +669,43 @@
         <v>6.9</v>
       </c>
       <c r="B6" t="n">
-        <v>4676</v>
+        <v>4777</v>
       </c>
       <c r="C6" t="n">
-        <v>1142</v>
+        <v>1226</v>
       </c>
       <c r="D6" t="n">
-        <v>1142</v>
+        <v>1226</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="G6" t="n">
-        <v>126</v>
+        <v>100</v>
       </c>
       <c r="H6" t="n">
-        <v>119</v>
+        <v>110</v>
       </c>
       <c r="I6" t="n">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="J6" t="n">
-        <v>63</v>
+        <v>50</v>
       </c>
       <c r="K6" t="n">
-        <v>37</v>
+        <v>56</v>
       </c>
       <c r="L6" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="M6" t="n">
-        <v>57</v>
+        <v>74</v>
       </c>
       <c r="N6" t="n">
-        <v>0.11</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="7">
@@ -713,43 +713,43 @@
         <v>8.300000000000001</v>
       </c>
       <c r="B7" t="n">
-        <v>4797</v>
+        <v>4638</v>
       </c>
       <c r="C7" t="n">
-        <v>1195</v>
+        <v>1219</v>
       </c>
       <c r="D7" t="n">
-        <v>1195</v>
+        <v>1219</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="G7" t="n">
-        <v>118</v>
+        <v>103</v>
       </c>
       <c r="H7" t="n">
-        <v>120</v>
+        <v>104</v>
       </c>
       <c r="I7" t="n">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="J7" t="n">
-        <v>46</v>
+        <v>70</v>
       </c>
       <c r="K7" t="n">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="L7" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="M7" t="n">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="N7" t="n">
-        <v>0.11</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="8">
@@ -757,40 +757,40 @@
         <v>9.699999999999999</v>
       </c>
       <c r="B8" t="n">
-        <v>4659</v>
+        <v>4597</v>
       </c>
       <c r="C8" t="n">
-        <v>1162</v>
+        <v>1184</v>
       </c>
       <c r="D8" t="n">
-        <v>1162</v>
+        <v>1184</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="G8" t="n">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="H8" t="n">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I8" t="n">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="J8" t="n">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="K8" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="L8" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M8" t="n">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="N8" t="n">
         <v>0.1</v>
@@ -801,40 +801,40 @@
         <v>11.3</v>
       </c>
       <c r="B9" t="n">
-        <v>4618</v>
+        <v>4656</v>
       </c>
       <c r="C9" t="n">
-        <v>1176</v>
+        <v>1141</v>
       </c>
       <c r="D9" t="n">
-        <v>1176</v>
+        <v>1141</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="G9" t="n">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="H9" t="n">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="I9" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J9" t="n">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="K9" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="L9" t="n">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="M9" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="N9" t="n">
         <v>0.11</v>

</xml_diff>